<commit_message>
feat: BART-MNLI pipeline, urgency detection, ratings, queue tracking, voice input, and symptom escalation re-routing
- Add BART-MNLI FastAPI sidecar (main.py rewrite) as switchable classifier alongside Gemini
- Add detectUrgency() for priority-based slot scheduling (routine/urgent/emergency)
- Add doctor ratings with recalculateDoctorRating() and /api/appointments/:id/rate endpoint
- Add live queue tracking via /api/queue/:doctorName/:date
- Add patient appointment cancellation and rescheduling endpoints
- Add voice input (Web Speech API) in app.js
- Add evaluation framework (evaluate.js + test_cases.json) comparing Gemini vs BART-MNLI
- Add urgency badges to doctor dashboard
- Fix symptom anchoring: detectSymptomEscalation() detects critical new symptoms mid-conversation,
  updates symptom profile, resets differential, and forces re-evaluation of specialist routing
- Fix specialty matching to use full symptomsSummary instead of only initial symptoms
</commit_message>
<xml_diff>
--- a/doctors.xlsx
+++ b/doctors.xlsx
@@ -436,7 +436,7 @@
         <v>mon 09:00-17:00, tue 09:00-17:00, wed 09:00-17:00, thu 09:00-17:00, fri 09:00-16:00</v>
       </c>
       <c r="F2" t="str">
-        <v>2026-06-09 14:30</v>
+        <v>2026-07-06 14:30</v>
       </c>
     </row>
     <row r="3">
@@ -456,7 +456,7 @@
         <v>mon 08:00-16:00, tue 08:00-16:00, wed 08:00-16:00, thu 08:00-16:00, fri 08:00-15:00</v>
       </c>
       <c r="F3" t="str">
-        <v>2026-06-10 12:30</v>
+        <v>2026-07-07 09:30</v>
       </c>
     </row>
     <row r="4">

</xml_diff>